<commit_message>
#93 Top board Completed #92 bottom board incomplete
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/Altium_Generated_BOM.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/Altium_Generated_BOM.xlsx
@@ -1086,10 +1086,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -1102,17 +1102,38 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1124,8 +1145,48 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1140,7 +1201,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1162,61 +1230,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1224,21 +1239,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1259,7 +1259,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1271,7 +1307,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1283,13 +1349,79 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1301,61 +1433,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1367,85 +1445,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1639,6 +1639,26 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -1659,45 +1679,6 @@
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1726,13 +1707,32 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF7F7F7F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1741,15 +1741,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1759,130 +1759,130 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="17" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="18" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="31" borderId="20" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="31" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>

<commit_message>
Top Board BOM finalized
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/Altium_Generated_BOM.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/Altium_Generated_BOM.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="346">
   <si>
     <t>Component list</t>
   </si>
@@ -304,7 +304,7 @@
     <t>CAP ALUM 220UF 20% 50V SMD</t>
   </si>
   <si>
-    <t>Cap Ceramic 0.1uF 50VDC X7R 10% SMD 0603 Paper T/R, CAP CER 0.1UF 100V X7R 0603</t>
+    <t>Cap Ceramic 0.1uF 50VDC X7R 10% SMD 0603 Paper T/R</t>
   </si>
   <si>
     <t>CAP CER 10000PF 25V X7R 0402</t>
@@ -325,7 +325,7 @@
     <t>CAP CER 0.082UF 50V X7R 0603</t>
   </si>
   <si>
-    <t>Cap Ceramic 0.22uF 100V X7R 10% SMD 0805 125°C Embossed T/R, CAP CER 220nF 35V 0805</t>
+    <t>Cap Ceramic 0.22uF 100V X7R 10% SMD 0805 125°C Embossed T/R, CAP CER 0.22UF 100V X7R 0805</t>
   </si>
   <si>
     <t>0603 .022uF 100volts X7R 10% T=0.8mm</t>
@@ -652,7 +652,7 @@
     <t>Manufacturer Part Number</t>
   </si>
   <si>
-    <t>CL10B104KB8NNNC, CC0603KRX7R0BB104</t>
+    <t>CL10B104KB8NNNC</t>
   </si>
   <si>
     <t>CC0402KRX7R8BB103</t>
@@ -673,7 +673,7 @@
     <t>CC0603KRX7R9BB823</t>
   </si>
   <si>
-    <t>08051C224K4T2A, GMK212BJ224KGHT</t>
+    <t>08051C224K4T2A</t>
   </si>
   <si>
     <t>CGA3E2X7R2A223K080AA</t>
@@ -808,7 +808,7 @@
     <t>Nichicon</t>
   </si>
   <si>
-    <t>Samsung, Yageo</t>
+    <t>Samsung</t>
   </si>
   <si>
     <t>Yageo</t>
@@ -820,7 +820,7 @@
     <t>Murata</t>
   </si>
   <si>
-    <t>Kyocera AVX, Taiyo Yuden</t>
+    <t>Kyocera AVX</t>
   </si>
   <si>
     <t>TDK</t>
@@ -829,16 +829,10 @@
     <t>Ymin</t>
   </si>
   <si>
-    <t>Samsung</t>
-  </si>
-  <si>
     <t>Wurth Electronics</t>
   </si>
   <si>
     <t>FH</t>
-  </si>
-  <si>
-    <t>Kyocera AVX</t>
   </si>
   <si>
     <t>Changzhou Huawei Elec</t>
@@ -2158,16 +2152,16 @@
         <v>257</v>
       </c>
       <c r="J9" s="30" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="K9" s="29" t="s">
+        <v>343</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>344</v>
+      </c>
+      <c r="M9" s="31" t="s">
         <v>345</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>346</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2194,7 +2188,7 @@
         <v>258</v>
       </c>
       <c r="J10" s="38" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K10" s="37">
         <v>1</v>
@@ -2202,7 +2196,7 @@
       <c r="L10" s="37"/>
       <c r="M10" s="41"/>
     </row>
-    <row r="11" spans="1:13" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="54">
         <f t="shared" ref="B11:B86" si="0">ROW(B11) - ROW($B$9)</f>
@@ -2226,7 +2220,7 @@
         <v>259</v>
       </c>
       <c r="J11" s="40" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K11" s="39">
         <v>13</v>
@@ -2258,7 +2252,7 @@
         <v>260</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="K12" s="37">
         <v>2</v>
@@ -2290,7 +2284,7 @@
         <v>261</v>
       </c>
       <c r="J13" s="40" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="K13" s="39">
         <v>1</v>
@@ -2322,7 +2316,7 @@
         <v>262</v>
       </c>
       <c r="J14" s="38" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="K14" s="37">
         <v>8</v>
@@ -2354,7 +2348,7 @@
         <v>260</v>
       </c>
       <c r="J15" s="40" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="K15" s="39">
         <v>3</v>
@@ -2386,7 +2380,7 @@
         <v>262</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K16" s="37">
         <v>6</v>
@@ -2418,7 +2412,7 @@
         <v>260</v>
       </c>
       <c r="J17" s="40" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="K17" s="39">
         <v>1</v>
@@ -2450,7 +2444,7 @@
         <v>263</v>
       </c>
       <c r="J18" s="38" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="K18" s="37">
         <v>8</v>
@@ -2482,7 +2476,7 @@
         <v>264</v>
       </c>
       <c r="J19" s="40" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="K19" s="39">
         <v>1</v>
@@ -2512,7 +2506,7 @@
         <v>265</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K20" s="37">
         <v>1</v>
@@ -2541,10 +2535,10 @@
       </c>
       <c r="H21" s="39"/>
       <c r="I21" s="39" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="K21" s="39">
         <v>2</v>
@@ -2576,7 +2570,7 @@
         <v>261</v>
       </c>
       <c r="J22" s="38" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="K22" s="37">
         <v>1</v>
@@ -2605,10 +2599,10 @@
       </c>
       <c r="H23" s="39"/>
       <c r="I23" s="39" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J23" s="40" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="K23" s="39">
         <v>1</v>
@@ -2637,10 +2631,10 @@
       </c>
       <c r="H24" s="37"/>
       <c r="I24" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J24" s="38" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="K24" s="37">
         <v>1</v>
@@ -2672,7 +2666,7 @@
         <v>260</v>
       </c>
       <c r="J25" s="40" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="K25" s="39">
         <v>1</v>
@@ -2701,10 +2695,10 @@
       </c>
       <c r="H26" s="37"/>
       <c r="I26" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J26" s="38" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="K26" s="37">
         <v>1</v>
@@ -2736,7 +2730,7 @@
         <v>262</v>
       </c>
       <c r="J27" s="40" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="K27" s="39">
         <v>1</v>
@@ -2765,10 +2759,10 @@
       </c>
       <c r="H28" s="37"/>
       <c r="I28" s="37" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="J28" s="38" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="K28" s="37">
         <v>1</v>
@@ -2795,10 +2789,10 @@
       <c r="G29" s="40"/>
       <c r="H29" s="39"/>
       <c r="I29" s="39" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="J29" s="40" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K29" s="39">
         <v>1</v>
@@ -2830,7 +2824,7 @@
         <v>260</v>
       </c>
       <c r="J30" s="38" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K30" s="37">
         <v>1</v>
@@ -2859,10 +2853,10 @@
       </c>
       <c r="H31" s="39"/>
       <c r="I31" s="39" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="J31" s="40" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K31" s="39">
         <v>4</v>
@@ -2891,7 +2885,7 @@
       </c>
       <c r="H32" s="37"/>
       <c r="I32" s="37" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="J32" s="38" t="s">
         <v>176</v>
@@ -2921,10 +2915,10 @@
       <c r="G33" s="40"/>
       <c r="H33" s="39"/>
       <c r="I33" s="39" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="J33" s="40" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K33" s="39">
         <v>1</v>
@@ -2951,10 +2945,10 @@
       <c r="G34" s="38"/>
       <c r="H34" s="37"/>
       <c r="I34" s="37" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="J34" s="38" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="K34" s="37">
         <v>2</v>
@@ -2983,7 +2977,7 @@
       </c>
       <c r="H35" s="39"/>
       <c r="I35" s="39" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="J35" s="40" t="s">
         <v>225</v>
@@ -3015,7 +3009,7 @@
       </c>
       <c r="H36" s="37"/>
       <c r="I36" s="37" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="J36" s="38" t="s">
         <v>179</v>
@@ -3079,7 +3073,7 @@
       </c>
       <c r="H38" s="37"/>
       <c r="I38" s="37" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="J38" s="38" t="s">
         <v>181</v>
@@ -3111,7 +3105,7 @@
       </c>
       <c r="H39" s="39"/>
       <c r="I39" s="39" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="J39" s="40" t="s">
         <v>182</v>
@@ -3143,7 +3137,7 @@
       </c>
       <c r="H40" s="37"/>
       <c r="I40" s="37" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="J40" s="38" t="s">
         <v>183</v>
@@ -3175,7 +3169,7 @@
       </c>
       <c r="H41" s="39"/>
       <c r="I41" s="39" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J41" s="40" t="s">
         <v>184</v>
@@ -3210,7 +3204,7 @@
         <v>264</v>
       </c>
       <c r="J42" s="38" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="K42" s="37">
         <v>1</v>
@@ -3237,10 +3231,10 @@
       </c>
       <c r="H43" s="39"/>
       <c r="I43" s="39" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="J43" s="40" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="K43" s="39">
         <v>1</v>
@@ -3269,7 +3263,7 @@
       </c>
       <c r="H44" s="37"/>
       <c r="I44" s="37" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J44" s="38" t="s">
         <v>186</v>
@@ -3301,7 +3295,7 @@
       </c>
       <c r="H45" s="39"/>
       <c r="I45" s="39" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J45" s="40" t="s">
         <v>227</v>
@@ -3333,7 +3327,7 @@
       </c>
       <c r="H46" s="37"/>
       <c r="I46" s="37" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J46" s="38" t="s">
         <v>188</v>
@@ -3364,7 +3358,7 @@
       <c r="H47" s="39"/>
       <c r="I47" s="39"/>
       <c r="J47" s="40" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="K47" s="39">
         <v>4</v>
@@ -3393,7 +3387,7 @@
       </c>
       <c r="H48" s="37"/>
       <c r="I48" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J48" s="38">
         <v>61300211121</v>
@@ -3425,7 +3419,7 @@
       </c>
       <c r="H49" s="39"/>
       <c r="I49" s="39" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J49" s="40" t="s">
         <v>191</v>
@@ -3460,7 +3454,7 @@
         <v>260</v>
       </c>
       <c r="J50" s="38" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="K50" s="37">
         <v>2</v>
@@ -3492,7 +3486,7 @@
         <v>260</v>
       </c>
       <c r="J51" s="40" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="K51" s="39">
         <v>1</v>
@@ -3521,10 +3515,10 @@
       </c>
       <c r="H52" s="37"/>
       <c r="I52" s="37" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J52" s="38" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="K52" s="37">
         <v>1</v>
@@ -3556,7 +3550,7 @@
         <v>260</v>
       </c>
       <c r="J53" s="40" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="K53" s="39">
         <v>2</v>
@@ -3588,7 +3582,7 @@
         <v>260</v>
       </c>
       <c r="J54" s="38" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="K54" s="37">
         <v>4</v>
@@ -3615,10 +3609,10 @@
       <c r="G55" s="40"/>
       <c r="H55" s="39"/>
       <c r="I55" s="39" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="J55" s="40" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="K55" s="39">
         <v>4</v>
@@ -3647,10 +3641,10 @@
       </c>
       <c r="H56" s="37"/>
       <c r="I56" s="37" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="J56" s="38" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="K56" s="37">
         <v>8</v>
@@ -3679,10 +3673,10 @@
       </c>
       <c r="H57" s="39"/>
       <c r="I57" s="39" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J57" s="40" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="K57" s="39">
         <v>1</v>
@@ -3714,7 +3708,7 @@
         <v>260</v>
       </c>
       <c r="J58" s="38" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K58" s="37">
         <v>1</v>
@@ -3743,10 +3737,10 @@
       </c>
       <c r="H59" s="39"/>
       <c r="I59" s="39" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J59" s="40" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="K59" s="39">
         <v>1</v>
@@ -3778,7 +3772,7 @@
         <v>260</v>
       </c>
       <c r="J60" s="38" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="K60" s="37">
         <v>1</v>
@@ -3807,10 +3801,10 @@
       </c>
       <c r="H61" s="39"/>
       <c r="I61" s="39" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J61" s="40" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K61" s="39">
         <v>1</v>
@@ -3842,7 +3836,7 @@
         <v>260</v>
       </c>
       <c r="J62" s="38" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="K62" s="37">
         <v>1</v>
@@ -3874,7 +3868,7 @@
         <v>260</v>
       </c>
       <c r="J63" s="40" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="K63" s="39">
         <v>1</v>
@@ -3906,7 +3900,7 @@
         <v>260</v>
       </c>
       <c r="J64" s="38" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="K64" s="37">
         <v>1</v>
@@ -3938,7 +3932,7 @@
         <v>260</v>
       </c>
       <c r="J65" s="40" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K65" s="39">
         <v>2</v>
@@ -3970,7 +3964,7 @@
         <v>260</v>
       </c>
       <c r="J66" s="38" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K66" s="37">
         <v>2</v>
@@ -3999,10 +3993,10 @@
       </c>
       <c r="H67" s="39"/>
       <c r="I67" s="39" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="J67" s="40" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K67" s="39">
         <v>1</v>
@@ -4034,7 +4028,7 @@
         <v>260</v>
       </c>
       <c r="J68" s="38" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K68" s="37">
         <v>2</v>
@@ -4063,10 +4057,10 @@
       </c>
       <c r="H69" s="39"/>
       <c r="I69" s="39" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J69" s="40" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K69" s="39">
         <v>1</v>
@@ -4095,10 +4089,10 @@
       </c>
       <c r="H70" s="37"/>
       <c r="I70" s="37" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="J70" s="38" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K70" s="37">
         <v>1</v>
@@ -4130,7 +4124,7 @@
         <v>260</v>
       </c>
       <c r="J71" s="40" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="K71" s="39">
         <v>6</v>
@@ -4157,10 +4151,10 @@
       <c r="G72" s="38"/>
       <c r="H72" s="37"/>
       <c r="I72" s="37" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="J72" s="38" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K72" s="37">
         <v>1</v>
@@ -4187,10 +4181,10 @@
       <c r="G73" s="40"/>
       <c r="H73" s="39"/>
       <c r="I73" s="39" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J73" s="40" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="K73" s="39">
         <v>1</v>
@@ -4245,7 +4239,7 @@
       <c r="G75" s="40"/>
       <c r="H75" s="39"/>
       <c r="I75" s="39" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J75" s="40" t="s">
         <v>196</v>
@@ -4277,7 +4271,7 @@
       </c>
       <c r="H76" s="37"/>
       <c r="I76" s="37" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J76" s="38">
         <v>750314597</v>
@@ -4309,7 +4303,7 @@
       </c>
       <c r="H77" s="39"/>
       <c r="I77" s="39" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J77" s="40" t="s">
         <v>197</v>
@@ -4341,7 +4335,7 @@
       </c>
       <c r="H78" s="37"/>
       <c r="I78" s="37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J78" s="38" t="s">
         <v>249</v>
@@ -4373,7 +4367,7 @@
       </c>
       <c r="H79" s="39"/>
       <c r="I79" s="39" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="J79" s="40" t="s">
         <v>250</v>
@@ -4405,7 +4399,7 @@
       </c>
       <c r="H80" s="37"/>
       <c r="I80" s="37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J80" s="38" t="s">
         <v>200</v>
@@ -4437,7 +4431,7 @@
       </c>
       <c r="H81" s="39"/>
       <c r="I81" s="39" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J81" s="40" t="s">
         <v>251</v>
@@ -4469,7 +4463,7 @@
       </c>
       <c r="H82" s="37"/>
       <c r="I82" s="37" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J82" s="38" t="s">
         <v>252</v>
@@ -4501,7 +4495,7 @@
       </c>
       <c r="H83" s="39"/>
       <c r="I83" s="39" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J83" s="40" t="s">
         <v>253</v>
@@ -4533,7 +4527,7 @@
       </c>
       <c r="H84" s="37"/>
       <c r="I84" s="37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J84" s="38" t="s">
         <v>254</v>
@@ -4565,7 +4559,7 @@
       </c>
       <c r="H85" s="39"/>
       <c r="I85" s="39" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J85" s="40" t="s">
         <v>204</v>
@@ -4597,7 +4591,7 @@
       </c>
       <c r="H86" s="37"/>
       <c r="I86" s="37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J86" s="38" t="s">
         <v>255</v>

</xml_diff>

<commit_message>
Top board 0.1uF caps added in BOM
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/Altium_Generated_BOM.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/Altium_Generated_BOM.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="344">
   <si>
     <t>Component list</t>
   </si>
@@ -70,7 +70,7 @@
     <t>C1</t>
   </si>
   <si>
-    <t>C2, C13, C15, C20, C40, C51, C52, C53, C54, C55, C61, CF1, CF2</t>
+    <t>C2, C13, C15, C20, C40, C51, C52, C53, C54, C55, C61, CF1, CF2, Cx1, Cx2</t>
   </si>
   <si>
     <t>C3, C46</t>
@@ -472,7 +472,7 @@
     <t>RES SMD 51R 100mW 0603</t>
   </si>
   <si>
-    <t>RES SMD 150 OHM 5% 1/20W 0201</t>
+    <t>RES SMD 150OHM 1/10W 0603</t>
   </si>
   <si>
     <t>RES SMD 2K OHM 1% 1/10W 0603</t>
@@ -589,6 +589,9 @@
     <t>SLF12575T-221M1R3-PF</t>
   </si>
   <si>
+    <t>PNLS5020-330</t>
+  </si>
+  <si>
     <t>LTST-G683GEBW</t>
   </si>
   <si>
@@ -613,9 +616,6 @@
     <t>RES 2512</t>
   </si>
   <si>
-    <t>Res-0201</t>
-  </si>
-  <si>
     <t>Solder Bridge</t>
   </si>
   <si>
@@ -709,9 +709,6 @@
     <t>PMEG3010EP,115</t>
   </si>
   <si>
-    <t>PNLS5020-330</t>
-  </si>
-  <si>
     <t>XZVG68W-2</t>
   </si>
   <si>
@@ -763,7 +760,7 @@
     <t>RC0603FR-0751RL</t>
   </si>
   <si>
-    <t>CRCW0201150RJNED</t>
+    <t>RC0603FR-07150RL</t>
   </si>
   <si>
     <t>RC0603FR-072KL</t>
@@ -884,9 +881,6 @@
   </si>
   <si>
     <t>Panasonic</t>
-  </si>
-  <si>
-    <t>Vishay Dale</t>
   </si>
   <si>
     <t>RALEC</t>
@@ -2146,22 +2140,22 @@
         <v>206</v>
       </c>
       <c r="H9" s="29" t="s">
+        <v>255</v>
+      </c>
+      <c r="I9" s="29" t="s">
         <v>256</v>
       </c>
-      <c r="I9" s="29" t="s">
-        <v>257</v>
-      </c>
       <c r="J9" s="30" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="K9" s="29" t="s">
+        <v>341</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>342</v>
+      </c>
+      <c r="M9" s="31" t="s">
         <v>343</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>344</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2185,10 +2179,10 @@
       </c>
       <c r="H10" s="37"/>
       <c r="I10" s="37" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J10" s="38" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="K10" s="37">
         <v>1</v>
@@ -2217,13 +2211,13 @@
       </c>
       <c r="H11" s="39"/>
       <c r="I11" s="39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J11" s="40" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="K11" s="39">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L11" s="39"/>
       <c r="M11" s="42"/>
@@ -2249,10 +2243,10 @@
       </c>
       <c r="H12" s="37"/>
       <c r="I12" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="K12" s="37">
         <v>2</v>
@@ -2281,10 +2275,10 @@
       </c>
       <c r="H13" s="39"/>
       <c r="I13" s="39" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J13" s="40" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K13" s="39">
         <v>1</v>
@@ -2313,10 +2307,10 @@
       </c>
       <c r="H14" s="37"/>
       <c r="I14" s="37" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J14" s="38" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="K14" s="37">
         <v>8</v>
@@ -2345,10 +2339,10 @@
       </c>
       <c r="H15" s="39"/>
       <c r="I15" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J15" s="40" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="K15" s="39">
         <v>3</v>
@@ -2377,10 +2371,10 @@
       </c>
       <c r="H16" s="37"/>
       <c r="I16" s="37" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="K16" s="37">
         <v>6</v>
@@ -2409,10 +2403,10 @@
       </c>
       <c r="H17" s="39"/>
       <c r="I17" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J17" s="40" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="K17" s="39">
         <v>1</v>
@@ -2441,10 +2435,10 @@
       </c>
       <c r="H18" s="37"/>
       <c r="I18" s="37" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J18" s="38" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="K18" s="37">
         <v>8</v>
@@ -2473,10 +2467,10 @@
       </c>
       <c r="H19" s="39"/>
       <c r="I19" s="39" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J19" s="40" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="K19" s="39">
         <v>1</v>
@@ -2503,10 +2497,10 @@
       <c r="G20" s="38"/>
       <c r="H20" s="37"/>
       <c r="I20" s="37" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="K20" s="37">
         <v>1</v>
@@ -2535,10 +2529,10 @@
       </c>
       <c r="H21" s="39"/>
       <c r="I21" s="39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J21" s="40" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="K21" s="39">
         <v>2</v>
@@ -2567,10 +2561,10 @@
       </c>
       <c r="H22" s="37"/>
       <c r="I22" s="37" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J22" s="38" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="K22" s="37">
         <v>1</v>
@@ -2599,10 +2593,10 @@
       </c>
       <c r="H23" s="39"/>
       <c r="I23" s="39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J23" s="40" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="K23" s="39">
         <v>1</v>
@@ -2631,10 +2625,10 @@
       </c>
       <c r="H24" s="37"/>
       <c r="I24" s="37" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J24" s="38" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="K24" s="37">
         <v>1</v>
@@ -2663,10 +2657,10 @@
       </c>
       <c r="H25" s="39"/>
       <c r="I25" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J25" s="40" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="K25" s="39">
         <v>1</v>
@@ -2695,10 +2689,10 @@
       </c>
       <c r="H26" s="37"/>
       <c r="I26" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J26" s="38" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="K26" s="37">
         <v>1</v>
@@ -2727,10 +2721,10 @@
       </c>
       <c r="H27" s="39"/>
       <c r="I27" s="39" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J27" s="40" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="K27" s="39">
         <v>1</v>
@@ -2759,10 +2753,10 @@
       </c>
       <c r="H28" s="37"/>
       <c r="I28" s="37" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J28" s="38" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="K28" s="37">
         <v>1</v>
@@ -2789,10 +2783,10 @@
       <c r="G29" s="40"/>
       <c r="H29" s="39"/>
       <c r="I29" s="39" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J29" s="40" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="K29" s="39">
         <v>1</v>
@@ -2821,10 +2815,10 @@
       </c>
       <c r="H30" s="37"/>
       <c r="I30" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J30" s="38" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="K30" s="37">
         <v>1</v>
@@ -2853,10 +2847,10 @@
       </c>
       <c r="H31" s="39"/>
       <c r="I31" s="39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J31" s="40" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K31" s="39">
         <v>4</v>
@@ -2885,7 +2879,7 @@
       </c>
       <c r="H32" s="37"/>
       <c r="I32" s="37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="J32" s="38" t="s">
         <v>176</v>
@@ -2915,10 +2909,10 @@
       <c r="G33" s="40"/>
       <c r="H33" s="39"/>
       <c r="I33" s="39" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J33" s="40" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="K33" s="39">
         <v>1</v>
@@ -2945,10 +2939,10 @@
       <c r="G34" s="38"/>
       <c r="H34" s="37"/>
       <c r="I34" s="37" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J34" s="38" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K34" s="37">
         <v>2</v>
@@ -2977,7 +2971,7 @@
       </c>
       <c r="H35" s="39"/>
       <c r="I35" s="39" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="J35" s="40" t="s">
         <v>225</v>
@@ -3009,7 +3003,7 @@
       </c>
       <c r="H36" s="37"/>
       <c r="I36" s="37" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J36" s="38" t="s">
         <v>179</v>
@@ -3041,7 +3035,7 @@
       </c>
       <c r="H37" s="39"/>
       <c r="I37" s="39" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J37" s="40" t="s">
         <v>180</v>
@@ -3073,7 +3067,7 @@
       </c>
       <c r="H38" s="37"/>
       <c r="I38" s="37" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J38" s="38" t="s">
         <v>181</v>
@@ -3105,7 +3099,7 @@
       </c>
       <c r="H39" s="39"/>
       <c r="I39" s="39" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J39" s="40" t="s">
         <v>182</v>
@@ -3137,7 +3131,7 @@
       </c>
       <c r="H40" s="37"/>
       <c r="I40" s="37" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J40" s="38" t="s">
         <v>183</v>
@@ -3169,7 +3163,7 @@
       </c>
       <c r="H41" s="39"/>
       <c r="I41" s="39" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J41" s="40" t="s">
         <v>184</v>
@@ -3201,10 +3195,10 @@
       </c>
       <c r="H42" s="37"/>
       <c r="I42" s="37" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J42" s="38" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="K42" s="37">
         <v>1</v>
@@ -3225,16 +3219,18 @@
       <c r="E43" s="40" t="s">
         <v>123</v>
       </c>
-      <c r="F43" s="39"/>
+      <c r="F43" s="39" t="s">
+        <v>186</v>
+      </c>
       <c r="G43" s="40" t="s">
-        <v>226</v>
+        <v>186</v>
       </c>
       <c r="H43" s="39"/>
       <c r="I43" s="39" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J43" s="40" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="K43" s="39">
         <v>1</v>
@@ -3256,17 +3252,17 @@
         <v>124</v>
       </c>
       <c r="F44" s="37" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G44" s="38" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H44" s="37"/>
       <c r="I44" s="37" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J44" s="38" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K44" s="37">
         <v>1</v>
@@ -3288,17 +3284,17 @@
         <v>125</v>
       </c>
       <c r="F45" s="39" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G45" s="40" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H45" s="39"/>
       <c r="I45" s="39" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J45" s="40" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="K45" s="39">
         <v>1</v>
@@ -3320,17 +3316,17 @@
         <v>126</v>
       </c>
       <c r="F46" s="37" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G46" s="38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H46" s="37"/>
       <c r="I46" s="37" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J46" s="38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K46" s="37">
         <v>2</v>
@@ -3352,13 +3348,13 @@
         <v>127</v>
       </c>
       <c r="F47" s="39" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G47" s="40"/>
       <c r="H47" s="39"/>
       <c r="I47" s="39"/>
       <c r="J47" s="40" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="K47" s="39">
         <v>4</v>
@@ -3380,14 +3376,14 @@
         <v>128</v>
       </c>
       <c r="F48" s="37" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G48" s="38">
         <v>61300211121</v>
       </c>
       <c r="H48" s="37"/>
       <c r="I48" s="37" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J48" s="38">
         <v>61300211121</v>
@@ -3412,17 +3408,17 @@
         <v>129</v>
       </c>
       <c r="F49" s="39" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G49" s="40" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H49" s="39"/>
       <c r="I49" s="39" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J49" s="40" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K49" s="39">
         <v>4</v>
@@ -3444,17 +3440,17 @@
         <v>130</v>
       </c>
       <c r="F50" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G50" s="38" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H50" s="37"/>
       <c r="I50" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J50" s="38" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="K50" s="37">
         <v>2</v>
@@ -3476,17 +3472,17 @@
         <v>131</v>
       </c>
       <c r="F51" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G51" s="40" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H51" s="39"/>
       <c r="I51" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J51" s="40" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="K51" s="39">
         <v>1</v>
@@ -3508,17 +3504,17 @@
         <v>132</v>
       </c>
       <c r="F52" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G52" s="38" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H52" s="37"/>
       <c r="I52" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J52" s="38" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="K52" s="37">
         <v>1</v>
@@ -3540,17 +3536,17 @@
         <v>133</v>
       </c>
       <c r="F53" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G53" s="40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H53" s="39"/>
       <c r="I53" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J53" s="40" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="K53" s="39">
         <v>2</v>
@@ -3572,17 +3568,17 @@
         <v>134</v>
       </c>
       <c r="F54" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G54" s="38" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H54" s="37"/>
       <c r="I54" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J54" s="38" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="K54" s="37">
         <v>4</v>
@@ -3604,15 +3600,15 @@
         <v>135</v>
       </c>
       <c r="F55" s="39" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G55" s="40"/>
       <c r="H55" s="39"/>
       <c r="I55" s="39" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J55" s="40" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="K55" s="39">
         <v>4</v>
@@ -3634,17 +3630,17 @@
         <v>136</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G56" s="38" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H56" s="37"/>
       <c r="I56" s="37" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J56" s="38" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="K56" s="37">
         <v>8</v>
@@ -3666,17 +3662,17 @@
         <v>137</v>
       </c>
       <c r="F57" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G57" s="40" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H57" s="39"/>
       <c r="I57" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J57" s="40" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="K57" s="39">
         <v>1</v>
@@ -3698,17 +3694,17 @@
         <v>138</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G58" s="38" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H58" s="37"/>
       <c r="I58" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J58" s="38" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="K58" s="37">
         <v>1</v>
@@ -3730,17 +3726,17 @@
         <v>139</v>
       </c>
       <c r="F59" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G59" s="40" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H59" s="39"/>
       <c r="I59" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J59" s="40" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="K59" s="39">
         <v>1</v>
@@ -3762,17 +3758,17 @@
         <v>140</v>
       </c>
       <c r="F60" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G60" s="38" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H60" s="37"/>
       <c r="I60" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J60" s="38" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K60" s="37">
         <v>1</v>
@@ -3794,17 +3790,17 @@
         <v>141</v>
       </c>
       <c r="F61" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G61" s="40" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H61" s="39"/>
       <c r="I61" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J61" s="40" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="K61" s="39">
         <v>1</v>
@@ -3826,17 +3822,17 @@
         <v>142</v>
       </c>
       <c r="F62" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G62" s="38" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H62" s="37"/>
       <c r="I62" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J62" s="38" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="K62" s="37">
         <v>1</v>
@@ -3858,17 +3854,17 @@
         <v>143</v>
       </c>
       <c r="F63" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G63" s="40" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H63" s="39"/>
       <c r="I63" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J63" s="40" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="K63" s="39">
         <v>1</v>
@@ -3890,17 +3886,17 @@
         <v>144</v>
       </c>
       <c r="F64" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G64" s="38" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H64" s="37"/>
       <c r="I64" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J64" s="38" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="K64" s="37">
         <v>1</v>
@@ -3922,17 +3918,17 @@
         <v>145</v>
       </c>
       <c r="F65" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G65" s="40" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H65" s="39"/>
       <c r="I65" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J65" s="40" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="K65" s="39">
         <v>2</v>
@@ -3954,17 +3950,17 @@
         <v>146</v>
       </c>
       <c r="F66" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G66" s="38" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H66" s="37"/>
       <c r="I66" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J66" s="38" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="K66" s="37">
         <v>2</v>
@@ -3986,17 +3982,17 @@
         <v>147</v>
       </c>
       <c r="F67" s="39" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G67" s="40" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H67" s="39"/>
       <c r="I67" s="39" t="s">
-        <v>285</v>
+        <v>259</v>
       </c>
       <c r="J67" s="40" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="K67" s="39">
         <v>1</v>
@@ -4018,17 +4014,17 @@
         <v>148</v>
       </c>
       <c r="F68" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G68" s="38" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H68" s="37"/>
       <c r="I68" s="37" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J68" s="38" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K68" s="37">
         <v>2</v>
@@ -4050,17 +4046,17 @@
         <v>149</v>
       </c>
       <c r="F69" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G69" s="40" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H69" s="39"/>
       <c r="I69" s="39" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J69" s="40" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="K69" s="39">
         <v>1</v>
@@ -4082,17 +4078,17 @@
         <v>150</v>
       </c>
       <c r="F70" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G70" s="38" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H70" s="37"/>
       <c r="I70" s="37" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J70" s="38" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K70" s="37">
         <v>1</v>
@@ -4114,17 +4110,17 @@
         <v>151</v>
       </c>
       <c r="F71" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G71" s="40" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H71" s="39"/>
       <c r="I71" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J71" s="40" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="K71" s="39">
         <v>6</v>
@@ -4146,15 +4142,15 @@
         <v>152</v>
       </c>
       <c r="F72" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G72" s="38"/>
       <c r="H72" s="37"/>
       <c r="I72" s="37" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J72" s="38" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K72" s="37">
         <v>1</v>
@@ -4176,15 +4172,15 @@
         <v>153</v>
       </c>
       <c r="F73" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G73" s="40"/>
       <c r="H73" s="39"/>
       <c r="I73" s="39" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J73" s="40" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="K73" s="39">
         <v>1</v>
@@ -4239,7 +4235,7 @@
       <c r="G75" s="40"/>
       <c r="H75" s="39"/>
       <c r="I75" s="39" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="J75" s="40" t="s">
         <v>196</v>
@@ -4271,7 +4267,7 @@
       </c>
       <c r="H76" s="37"/>
       <c r="I76" s="37" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J76" s="38">
         <v>750314597</v>
@@ -4303,7 +4299,7 @@
       </c>
       <c r="H77" s="39"/>
       <c r="I77" s="39" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J77" s="40" t="s">
         <v>197</v>
@@ -4331,14 +4327,14 @@
         <v>198</v>
       </c>
       <c r="G78" s="38" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H78" s="37"/>
       <c r="I78" s="37" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J78" s="38" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K78" s="37">
         <v>1</v>
@@ -4363,14 +4359,14 @@
         <v>199</v>
       </c>
       <c r="G79" s="40" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H79" s="39"/>
       <c r="I79" s="39" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J79" s="40" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K79" s="39">
         <v>1</v>
@@ -4399,7 +4395,7 @@
       </c>
       <c r="H80" s="37"/>
       <c r="I80" s="37" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J80" s="38" t="s">
         <v>200</v>
@@ -4427,14 +4423,14 @@
         <v>201</v>
       </c>
       <c r="G81" s="40" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H81" s="39"/>
       <c r="I81" s="39" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J81" s="40" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="K81" s="39">
         <v>1</v>
@@ -4459,14 +4455,14 @@
         <v>202</v>
       </c>
       <c r="G82" s="38" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H82" s="37"/>
       <c r="I82" s="37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J82" s="38" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="K82" s="37">
         <v>1</v>
@@ -4491,14 +4487,14 @@
         <v>203</v>
       </c>
       <c r="G83" s="40" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H83" s="39"/>
       <c r="I83" s="39" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="J83" s="40" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="K83" s="39">
         <v>1</v>
@@ -4523,14 +4519,14 @@
         <v>201</v>
       </c>
       <c r="G84" s="38" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H84" s="37"/>
       <c r="I84" s="37" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J84" s="38" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="K84" s="37">
         <v>2</v>
@@ -4559,7 +4555,7 @@
       </c>
       <c r="H85" s="39"/>
       <c r="I85" s="39" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J85" s="40" t="s">
         <v>204</v>
@@ -4587,14 +4583,14 @@
         <v>205</v>
       </c>
       <c r="G86" s="38" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H86" s="37"/>
       <c r="I86" s="37" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J86" s="38" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="K86" s="37">
         <v>1</v>

</xml_diff>